<commit_message>
fix(templates): sanitize default cell values to '-' in GranSuelo and GranAgregado templates
</commit_message>
<xml_diff>
--- a/app/templates/Subir auditoria/1-INF.-N-000-26-SU24-GRA.-S.-V09.xlsx
+++ b/app/templates/Subir auditoria/1-INF.-N-000-26-SU24-GRA.-S.-V09.xlsx
@@ -21694,7 +21694,11 @@
       <c r="G11" s="780"/>
       <c r="H11" s="779"/>
       <c r="I11" s="780"/>
-      <c r="J11" s="682"/>
+      <c r="J11" s="682" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="K11" s="386"/>
       <c r="L11" s="681"/>
       <c r="M11" s="681"/>
@@ -22776,8 +22780,10 @@
       <c r="Q2" s="323" t="s">
         <v>362</v>
       </c>
-      <c r="R2" s="529" t="s">
-        <v>442</v>
+      <c r="R2" s="529" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="S2" s="385"/>
       <c r="T2" s="279"/>
@@ -22801,15 +22807,19 @@
       <c r="Q3" s="323" t="s">
         <v>363</v>
       </c>
-      <c r="R3" s="529" t="s">
-        <v>442</v>
+      <c r="R3" s="529" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="S3" s="385"/>
       <c r="U3" s="560" t="s">
         <v>467</v>
       </c>
-      <c r="V3" s="540" t="s">
-        <v>442</v>
+      <c r="V3" s="540" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="W3" s="284">
         <f>+FORMATO!J11</f>

</xml_diff>